<commit_message>
fix(flipkart-recon): scope Phase 3 reconciliation audit to April 2026 only
- Auto-detect April settlements batch (d2263c38, 529 rows) via settlement_date
- all_order_item_ids() now accepts settlements_batch_id to restrict scope
- reconcile_order() passes batch_id to settlement lookup (no May rows mixed in)
- Result: 758 orders (621 Apr orders + 137 Apr-settlement-only), MATCHED=170,
  OVER_PAID=98, RETURN_RECOVERY=69, MISSING_FEE_RECORD=43, MISSING_SETTLEMENT=378
- 378 MISSING_SETTLEMENT is expected: Apr orders settled in May cycle
- Zero leakage, zero SHORT_PAID

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clearsettle-app/microservices/flipkart_reconciliation/tests/reconciliation/recon_audit_reports/16_test_suite_report.xlsx
+++ b/clearsettle-app/microservices/flipkart_reconciliation/tests/reconciliation/recon_audit_reports/16_test_suite_report.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Orders with no order record: 346, Settled orders without fee: 444, Orders without settlement: 39</t>
+          <t>Orders with no order record: 138, Settled orders without fee: 134, Orders without settlement: 378</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Verified formula for 927 orders</t>
+          <t>Verified formula for 380 orders</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MATCHED=398, SHORT_PAID=0, OVER_PAID=198, RETURN_RECOVERY=157, MISSING_SETTLEMENT=39, MISSING_FEE_RECORD=174. Match rate: 41.0%. Net diff: Rs.494.71</t>
+          <t>MATCHED=170, SHORT_PAID=0, OVER_PAID=98, RETURN_RECOVERY=69, MISSING_SETTLEMENT=378, MISSING_FEE_RECORD=43. Match rate: 22.4%. Net diff: Rs.2347.95</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Avg=74.2%, High=439, Medium=146, Low=385</t>
+          <t>Avg=75.7%, High=202, Medium=319, Low=237</t>
         </is>
       </c>
     </row>

</xml_diff>